<commit_message>
CSV en LF et non CRLF, plus un controle au niveau octet
Le modele officiel confirme l'en-tete, le separateur et single_chain. Mais la
comparaison octet par octet a montre que mon fichier etait en CRLF : le
csv.writer de Python ecrit \r\n par defaut. Conforme RFC 4180 et lu par
pandas, mais un parseur qui decoupe sur \n sans nettoyer lit
molecule_class = "single_chain\r" et le trouve hors enumeration. Panne
silencieuse sur le champ precisement en cause.

- lineterminator="\n" dans build_submission.py et build_metadata_package.py
- bytes_check() ajoute comme 9e controle : en-tete exact, BOM, CR,
  guillemets, newline finale, nombre de champs par ligne

Le controle precedent affirmait LF a tort : il cherchait le mot CRLF dans la
sortie de `file`, qui ne le mentionne pas sur macOS, donc il ne pouvait pas
echouer. Un controle qui ne peut pas echouer n'est pas un controle.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/egfr_analysis_working_copy.xlsx
+++ b/docs/egfr_analysis_working_copy.xlsx
@@ -29,7 +29,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Geometrie mutants'!$A$1:$Q$37</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Orthogonal detail'!$A$1:$K$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Methode et limites'!$A$1:$B$18</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Controles'!$A$1:$C$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Controles'!$A$1:$C$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Ecartes et motifs'!$A$1:$H$30</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1656,7 +1656,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -1817,9 +1817,26 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>octets : en-tete exact, BOM, CRLF, guillemets, champs</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>en-tete exact, pas de BOM, LF, 6 lignes de donnees a 3 champs</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:C9"/>
-  <conditionalFormatting sqref="B2:B9">
+  <autoFilter ref="A1:C10"/>
+  <conditionalFormatting sqref="B2:B10">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"OK"</formula>
     </cfRule>

</xml_diff>

<commit_message>
Controle de nouveaute : fd5dae..._seq1 refuse a 2/4, son frere le remplace
Proteinbase exige un score de nouveaute de 3/4 minimum. fd5dae7987a2388d_seq1
sort a 2/4. Le refus est inscrit comme regle NOVELTY_REJECTED plutot que par
un retrait manuel, ce qui laisse la regle « un design par squelette » reprendre
le frere seq0 : meme squelette, sequence differente a 24 %, metriques quasi
identiques. 6 designs sur 6 squelettes, controle negatif toujours au rang 6,
9 controles passes.

FAUX MOTIF RATTRAPE AVANT ENVOI : DESIGN_METRICS.md annoncait pour seq1 « a
design on the same backbone ranked higher », ce qui est faux — seq1 etait mieux
classe que son remplacant, c'est la plateforme qui l'a ecarte. Un motif errone
dans la table de l'entonnoir aurait ruine ce a quoi elle sert.
build_metrics_markdown.py importe desormais NOVELTY_REJECTED depuis
build_submission.py pour que les deux ne puissent pas diverger.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/egfr_analysis_working_copy.xlsx
+++ b/docs/egfr_analysis_working_copy.xlsx
@@ -1315,12 +1315,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>egfr-dIII-prod02_denovo_l58_fd5dae7987a2388d_seq1</t>
+          <t>egfr-dIII-prod02_denovo_l58_fd5dae7987a2388d_seq0</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1340,7 +1340,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-8.0</t>
+          <t>-11.0</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -1360,22 +1360,22 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>0.956</t>
+          <t>0.993</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>-0.07</t>
+          <t>-0.01</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>-0.12</t>
+          <t>-0.11</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>-0.13</t>
+          <t>-2.65</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -1385,17 +1385,17 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>0.938</t>
+          <t>0.944</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>0.002</t>
+          <t>0.007</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>0.812</t>
+          <t>0.806</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
@@ -1405,17 +1405,17 @@
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>3.31</t>
+          <t>3.36</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>159.9</t>
+          <t>147.1</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>0.778</t>
+          <t>0.789</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
@@ -1430,7 +1430,7 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>916.6</t>
+          <t>885.6</t>
         </is>
       </c>
       <c r="Y6" t="inlineStr">
@@ -1440,7 +1440,7 @@
       </c>
       <c r="Z6" t="inlineStr">
         <is>
-          <t>0.39</t>
+          <t>0.37</t>
         </is>
       </c>
       <c r="AA6" t="inlineStr">
@@ -1450,12 +1450,12 @@
       </c>
       <c r="AB6" t="inlineStr">
         <is>
-          <t>0.938</t>
+          <t>0.887</t>
         </is>
       </c>
       <c r="AC6" t="inlineStr">
         <is>
-          <t>0.936</t>
+          <t>0.937</t>
         </is>
       </c>
       <c r="AD6" t="inlineStr"/>
@@ -1466,7 +1466,7 @@
       </c>
       <c r="AF6" t="inlineStr">
         <is>
-          <t>IEVDENLPAHEQVFKILEEGTRKEFEARRAGKEEEAERISEEAVKKIEEIFEKEKNPE</t>
+          <t>IEVDPNLPVHEQVFLILEKGTKAEFEALRAGNEKEAEEISKEAVEKIEEAFEKEENPE</t>
         </is>
       </c>
     </row>
@@ -1728,7 +1728,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>20.7% entre 59_36dbfc4737a3e59b_seq1 et 58_fd5dae7987a2388d_seq1</t>
+          <t>20.3% entre 59_36dbfc4737a3e59b_seq1 et 61_cd272a8fd929c7ee_seq0</t>
         </is>
       </c>
     </row>
@@ -1912,29 +1912,25 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>egfr-dIII-prod02_denovo_l62_a6d2f6834f22e574_seq1__S44D</t>
+          <t>egfr-dIII-prod02_denovo_l58_fd5dae7987a2388d_seq1</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>a6d2f6834f22e574</t>
+          <t>fd5dae7987a2388d</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>mutant</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>S44D</t>
-        </is>
-      </c>
+          <t>bindcraft</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
           <t>absent</t>
@@ -1942,37 +1938,41 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>VERT</t>
+          <t>sans objet</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>mutant non eligible : mecanisme_robustesse='neutre' attendu 'robuste'</t>
+          <t>refuse par le controle de nouveaute de la plateforme (score 2/4, minimum requis 3/4)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>egfr-dIII-prod02_denovo_l92_5c3ec1903e03c261_seq1</t>
+          <t>egfr-dIII-prod02_denovo_l62_a6d2f6834f22e574_seq1__S44D</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>5c3ec1903e03c261</t>
+          <t>a6d2f6834f22e574</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>bindcraft</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr"/>
+          <t>mutant</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>S44D</t>
+        </is>
+      </c>
       <c r="F3" t="inlineStr">
         <is>
           <t>absent</t>
@@ -1980,29 +1980,29 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>sans objet</t>
+          <t>VERT</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>palier pH ecarte : contre-selectif — la liaison est predite DEFAVORISEE a pH 6,5, soit l'inverse du critere de rang le plus eleve du challenge</t>
+          <t>mutant non eligible : mecanisme_robustesse='neutre' attendu 'robuste'</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>egfr-dIII-prod02_denovo_l62_a6d2f6834f22e574_seq1</t>
+          <t>egfr-dIII-prod02_denovo_l92_5c3ec1903e03c261_seq1</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>a6d2f6834f22e574</t>
+          <t>5c3ec1903e03c261</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -2030,17 +2030,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>14</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>egfr-dIII-prod02_denovo_l92_5c3ec1903e03c261_seq0</t>
+          <t>egfr-dIII-prod02_denovo_l62_a6d2f6834f22e574_seq1</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>5c3ec1903e03c261</t>
+          <t>a6d2f6834f22e574</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -2068,17 +2068,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>egfr-dIII-prod02_denovo_l64_4a818d7951649b77_seq0</t>
+          <t>egfr-dIII-prod02_denovo_l92_5c3ec1903e03c261_seq0</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>4a818d7951649b77</t>
+          <t>5c3ec1903e03c261</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -2106,17 +2106,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>egfr-dIII-prod02_denovo_l61_a6334a3a912c86f1_seq0</t>
+          <t>egfr-dIII-prod02_denovo_l64_4a818d7951649b77_seq0</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>a6334a3a912c86f1</t>
+          <t>4a818d7951649b77</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -2144,17 +2144,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>17</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>egfr-dIII-prod01_denovo_l64_1e7ab6d8f00c9958_seq0</t>
+          <t>egfr-dIII-prod02_denovo_l61_a6334a3a912c86f1_seq0</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>1e7ab6d8f00c9958</t>
+          <t>a6334a3a912c86f1</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -2182,17 +2182,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>18</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>egfr-dIII-prod02_denovo_l62_a6d2f6834f22e574_seq0</t>
+          <t>egfr-dIII-prod01_denovo_l64_1e7ab6d8f00c9958_seq0</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>a6d2f6834f22e574</t>
+          <t>1e7ab6d8f00c9958</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -2220,17 +2220,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>19</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>egfr-dIII-prod02_denovo_l61_a6334a3a912c86f1_seq1</t>
+          <t>egfr-dIII-prod02_denovo_l62_a6d2f6834f22e574_seq0</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>a6334a3a912c86f1</t>
+          <t>a6d2f6834f22e574</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -2258,17 +2258,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>20</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>egfr-dIII-prod02_denovo_l73_5b295c4d9e1ff73f_seq0</t>
+          <t>egfr-dIII-prod02_denovo_l61_a6334a3a912c86f1_seq1</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>5b295c4d9e1ff73f</t>
+          <t>a6334a3a912c86f1</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -2296,17 +2296,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>21</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>egfr-dIII-prod02_denovo_l64_4a818d7951649b77_seq1</t>
+          <t>egfr-dIII-prod02_denovo_l73_5b295c4d9e1ff73f_seq0</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>4a818d7951649b77</t>
+          <t>5b295c4d9e1ff73f</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -2334,17 +2334,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>22</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>egfr-dIII-prod02_denovo_l73_5b295c4d9e1ff73f_seq1</t>
+          <t>egfr-dIII-prod02_denovo_l64_4a818d7951649b77_seq1</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>5b295c4d9e1ff73f</t>
+          <t>4a818d7951649b77</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -2372,17 +2372,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>23</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>egfr-dIII-prod01_denovo_l55_f6d5f550a210fd48_seq0</t>
+          <t>egfr-dIII-prod02_denovo_l73_5b295c4d9e1ff73f_seq1</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>f6d5f550a210fd48</t>
+          <t>5b295c4d9e1ff73f</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -2410,12 +2410,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>24</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>egfr-dIII-prod01_denovo_l55_f6d5f550a210fd48_seq0__S38D</t>
+          <t>egfr-dIII-prod01_denovo_l55_f6d5f550a210fd48_seq0</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2425,22 +2425,18 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>mutant</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>S38D</t>
-        </is>
-      </c>
+          <t>bindcraft</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
-          <t>INDETERMINE</t>
+          <t>absent</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>INDETERMINE</t>
+          <t>sans objet</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -2452,17 +2448,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>25</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>egfr-dIII-prod02_denovo_l73_5b295c4d9e1ff73f_seq1__H23E</t>
+          <t>egfr-dIII-prod01_denovo_l55_f6d5f550a210fd48_seq0__S38D</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>5b295c4d9e1ff73f</t>
+          <t>f6d5f550a210fd48</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -2472,12 +2468,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>H23E</t>
+          <t>S38D</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>absent</t>
+          <t>INDETERMINE</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -2494,12 +2490,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>26</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>egfr-dIII-prod02_denovo_l73_5b295c4d9e1ff73f_seq0__H23E</t>
+          <t>egfr-dIII-prod02_denovo_l73_5b295c4d9e1ff73f_seq1__H23E</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2536,17 +2532,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>27</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>egfr-dIII-prod02_denovo_l64_4a818d7951649b77_seq0__P39D</t>
+          <t>egfr-dIII-prod02_denovo_l73_5b295c4d9e1ff73f_seq0__H23E</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>4a818d7951649b77</t>
+          <t>5b295c4d9e1ff73f</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -2556,7 +2552,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>P39D</t>
+          <t>H23E</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -2566,7 +2562,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>VERT</t>
+          <t>INDETERMINE</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -2578,17 +2574,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>28</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>egfr-dIII-prod02_denovo_l61_cd272a8fd929c7ee_seq1__N21E</t>
+          <t>egfr-dIII-prod02_denovo_l64_4a818d7951649b77_seq0__P39D</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>cd272a8fd929c7ee</t>
+          <t>4a818d7951649b77</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -2598,7 +2594,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>N21E</t>
+          <t>P39D</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -2608,24 +2604,24 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>ROUGE</t>
+          <t>VERT</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>mutant non eligible : mecanisme_robustesse='neutre' attendu 'robuste' ; verdict_carboxylate='ROUGE' attendu 'VERT'</t>
+          <t>palier pH ecarte : contre-selectif — la liaison est predite DEFAVORISEE a pH 6,5, soit l'inverse du critere de rang le plus eleve du challenge</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>29</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>egfr-dIII-prod02_denovo_l61_cd272a8fd929c7ee_seq0__N21E</t>
+          <t>egfr-dIII-prod02_denovo_l61_cd272a8fd929c7ee_seq1__N21E</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2662,17 +2658,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>30</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>egfr-dIII-prod01_denovo_l64_1e7ab6d8f00c9958_seq0__S28D</t>
+          <t>egfr-dIII-prod02_denovo_l61_cd272a8fd929c7ee_seq0__N21E</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>1e7ab6d8f00c9958</t>
+          <t>cd272a8fd929c7ee</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -2682,39 +2678,39 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>S28D</t>
+          <t>N21E</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>INDETERMINE</t>
+          <t>absent</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>INDETERMINE</t>
+          <t>ROUGE</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>palier pH ecarte : contre-selectif — la liaison est predite DEFAVORISEE a pH 6,5, soit l'inverse du critere de rang le plus eleve du challenge</t>
+          <t>mutant non eligible : mecanisme_robustesse='neutre' attendu 'robuste' ; verdict_carboxylate='ROUGE' attendu 'VERT'</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>31</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>egfr-dIII-prod02_denovo_l62_a6d2f6834f22e574_seq0__S44D</t>
+          <t>egfr-dIII-prod01_denovo_l64_1e7ab6d8f00c9958_seq0__S28D</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>a6d2f6834f22e574</t>
+          <t>1e7ab6d8f00c9958</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -2724,7 +2720,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>S44D</t>
+          <t>S28D</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -2746,17 +2742,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>32</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>egfr-dIII-prod02_denovo_l61_a6334a3a912c86f1_seq0__S15D</t>
+          <t>egfr-dIII-prod02_denovo_l62_a6d2f6834f22e574_seq0__S44D</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>a6334a3a912c86f1</t>
+          <t>a6d2f6834f22e574</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -2766,17 +2762,17 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>S15D</t>
+          <t>S44D</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>absent</t>
+          <t>INDETERMINE</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>ROUGE</t>
+          <t>INDETERMINE</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -2788,12 +2784,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>33</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>egfr-dIII-prod02_denovo_l61_a6334a3a912c86f1_seq1__S15D</t>
+          <t>egfr-dIII-prod02_denovo_l61_a6334a3a912c86f1_seq0__S15D</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -2813,7 +2809,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>INDETERMINE</t>
+          <t>absent</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -2830,17 +2826,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>34</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>egfr-dIII-prod02_denovo_l64_4a818d7951649b77_seq1__F38D</t>
+          <t>egfr-dIII-prod02_denovo_l61_a6334a3a912c86f1_seq1__S15D</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>4a818d7951649b77</t>
+          <t>a6334a3a912c86f1</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -2850,12 +2846,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>F38D</t>
+          <t>S15D</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>absent</t>
+          <t>INDETERMINE</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -2872,25 +2868,29 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>35</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>egfr-dIII-prod02_denovo_l63_987fe804e455bc58_seq0</t>
+          <t>egfr-dIII-prod02_denovo_l64_4a818d7951649b77_seq1__F38D</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>987fe804e455bc58</t>
+          <t>4a818d7951649b77</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>bindcraft</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr"/>
+          <t>mutant</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>F38D</t>
+        </is>
+      </c>
       <c r="F26" t="inlineStr">
         <is>
           <t>absent</t>
@@ -2898,29 +2898,29 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>sans objet</t>
+          <t>ROUGE</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>squelette deja represente par un design mieux classe</t>
+          <t>palier pH ecarte : contre-selectif — la liaison est predite DEFAVORISEE a pH 6,5, soit l'inverse du critere de rang le plus eleve du challenge</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>egfr-dIII-prod02_denovo_l61_cd272a8fd929c7ee_seq1</t>
+          <t>egfr-dIII-prod02_denovo_l63_987fe804e455bc58_seq0</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>cd272a8fd929c7ee</t>
+          <t>987fe804e455bc58</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -2948,17 +2948,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>egfr-dIII-prod02_denovo_l59_36dbfc4737a3e59b_seq0</t>
+          <t>egfr-dIII-prod02_denovo_l61_cd272a8fd929c7ee_seq1</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>36dbfc4737a3e59b</t>
+          <t>cd272a8fd929c7ee</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -2986,17 +2986,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>egfr-dIII-prod02_denovo_l58_fd5dae7987a2388d_seq0</t>
+          <t>egfr-dIII-prod02_denovo_l59_36dbfc4737a3e59b_seq0</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>fd5dae7987a2388d</t>
+          <t>36dbfc4737a3e59b</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">

</xml_diff>